<commit_message>
Modified path to be relative
</commit_message>
<xml_diff>
--- a/Rules/rules.xlsx
+++ b/Rules/rules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EstebanDavyt\Desktop\PythonScript\Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B61A25BE-6D39-460D-91F8-0A1AB651B189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64332042-D3EF-4B1A-8E97-29F2A63A8C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="17820" windowHeight="17505" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
+    <workbookView xWindow="4890" yWindow="2280" windowWidth="21600" windowHeight="7815" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
   <si>
     <t>FormNumber</t>
   </si>
@@ -183,9 +183,6 @@
   </si>
   <si>
     <t>CA</t>
-  </si>
-  <si>
-    <t>Number Of Spaces</t>
   </si>
 </sst>
 </file>
@@ -593,469 +590,435 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5CE7AC6-E3FE-4E27-912C-E07231E907AF}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="6">
+        <v>41727</v>
+      </c>
+      <c r="C2" s="6">
+        <v>2958101</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="5">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>3</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="6">
-        <v>41727</v>
-      </c>
-      <c r="D2" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="5">
-        <v>1</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="5">
-        <v>10</v>
-      </c>
+      <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
+      <c r="B3" s="6">
+        <v>1</v>
+      </c>
       <c r="C3" s="6">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6">
         <v>2958101</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="E3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="5">
-        <v>1</v>
-      </c>
-      <c r="J3" s="5" t="s">
+      <c r="H3" s="5">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>16</v>
       </c>
+      <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="5">
+      <c r="L3" s="5">
         <v>15</v>
       </c>
+      <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="B4" s="6">
+        <v>43871</v>
+      </c>
       <c r="C4" s="6">
-        <v>43871</v>
-      </c>
-      <c r="D4" s="6">
         <v>2958465</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="E4" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="5">
-        <v>1</v>
-      </c>
-      <c r="J4" s="5" t="s">
+      <c r="H4" s="5">
+        <v>1</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="5">
+      <c r="L4" s="5">
         <v>31</v>
       </c>
+      <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>29</v>
       </c>
+      <c r="B5" s="6">
+        <v>45608</v>
+      </c>
       <c r="C5" s="6">
-        <v>45608</v>
-      </c>
-      <c r="D5" s="6">
         <v>2958101</v>
       </c>
+      <c r="D5" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="E5" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="5">
-        <v>1</v>
-      </c>
-      <c r="J5" s="5" t="s">
+      <c r="H5" s="5">
+        <v>1</v>
+      </c>
+      <c r="I5" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="5">
+      <c r="L5" s="5">
         <v>50</v>
       </c>
+      <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
+      <c r="B6" s="6">
+        <v>1</v>
+      </c>
       <c r="C6" s="6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6">
         <v>2958101</v>
       </c>
+      <c r="D6" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="E6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="5">
-        <v>1</v>
-      </c>
-      <c r="J6" s="5" t="s">
+      <c r="H6" s="5">
+        <v>1</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="5">
+      <c r="L6" s="5">
         <v>60</v>
       </c>
+      <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>2</v>
-      </c>
-      <c r="B7" s="5" t="s">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>35</v>
       </c>
+      <c r="B7" s="6">
+        <v>1</v>
+      </c>
       <c r="C7" s="6">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6">
         <v>2958101</v>
       </c>
+      <c r="D7" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="E7" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="5">
-        <v>1</v>
-      </c>
-      <c r="J7" s="5" t="s">
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J7" s="4"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="5">
+      <c r="L7" s="5">
         <v>70</v>
       </c>
+      <c r="M7" s="4"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8" s="5" t="s">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>38</v>
       </c>
+      <c r="B8" s="6">
+        <v>1</v>
+      </c>
       <c r="C8" s="6">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6">
         <v>2958101</v>
       </c>
+      <c r="D8" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="E8" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="5">
+      <c r="H8" s="5">
         <v>0</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J8" s="4"/>
       <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="5">
+      <c r="L8" s="5">
         <v>80</v>
       </c>
+      <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>2</v>
-      </c>
-      <c r="B9" s="5" t="s">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>41</v>
       </c>
+      <c r="B9" s="7">
+        <v>43857</v>
+      </c>
       <c r="C9" s="7">
-        <v>43857</v>
-      </c>
-      <c r="D9" s="7">
         <v>2958465</v>
       </c>
+      <c r="D9" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="E9" s="5" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="5">
+      <c r="H9" s="5">
         <v>0</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J9" s="4"/>
       <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="5">
+      <c r="L9" s="5">
         <v>83</v>
       </c>
+      <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10" s="5" t="s">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>43</v>
       </c>
+      <c r="B10" s="6">
+        <v>1</v>
+      </c>
       <c r="C10" s="6">
-        <v>1</v>
-      </c>
-      <c r="D10" s="6">
         <v>2958101</v>
       </c>
+      <c r="D10" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="E10" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="5">
+      <c r="H10" s="5">
         <v>0</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="J10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="5">
+      <c r="L10" s="5">
         <v>85</v>
       </c>
+      <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>3</v>
-      </c>
-      <c r="B11" s="5" t="s">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>45</v>
       </c>
+      <c r="B11" s="6">
+        <v>44574</v>
+      </c>
       <c r="C11" s="6">
-        <v>44574</v>
-      </c>
-      <c r="D11" s="6">
         <v>2958101</v>
       </c>
+      <c r="D11" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="E11" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="H11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="5">
-        <v>1</v>
-      </c>
-      <c r="J11" s="5" t="s">
+      <c r="H11" s="5">
+        <v>1</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M11" s="5">
+      <c r="L11" s="5">
         <v>10120</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added wholesale info to document and filedocument generator
</commit_message>
<xml_diff>
--- a/Rules/rules.xlsx
+++ b/Rules/rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EstebanDavyt\Desktop\PythonScript\Rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JuanCoates\OneDrive - Combined Ratio\Desktop\forms script\PythonScript\Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64332042-D3EF-4B1A-8E97-29F2A63A8C3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E5266F-2248-4879-9FA8-1C0F368D6F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4890" yWindow="2280" windowWidth="21600" windowHeight="7815" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
+    <workbookView xWindow="-3510" yWindow="4095" windowWidth="19380" windowHeight="11175" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>FormNumber</t>
   </si>
@@ -86,9 +86,6 @@
     <t>ALL</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
     <t>IL 00 17</t>
   </si>
   <si>
@@ -104,92 +101,20 @@
     <t>C</t>
   </si>
   <si>
-    <t>HUD AA 0014</t>
-  </si>
-  <si>
-    <t>02 12</t>
-  </si>
-  <si>
-    <t>Florida Policyholder Notice</t>
-  </si>
-  <si>
-    <t>FL</t>
-  </si>
-  <si>
-    <t>IL P 001</t>
-  </si>
-  <si>
-    <t>01 04</t>
-  </si>
-  <si>
-    <t>U.S. Treasury Departments (OFAC) Advisory Notice</t>
-  </si>
-  <si>
-    <t>HUD-IL 1002</t>
-  </si>
-  <si>
-    <t>09 24</t>
-  </si>
-  <si>
-    <t>Privacy Notice</t>
-  </si>
-  <si>
-    <t>IL 00 21</t>
-  </si>
-  <si>
-    <t>09 08</t>
-  </si>
-  <si>
-    <t>Nuclear Energy Liability Exclusion Endorsement</t>
-  </si>
-  <si>
-    <t>HUD-IL 2001</t>
-  </si>
-  <si>
-    <t>09 12</t>
-  </si>
-  <si>
-    <t>Minimum Policy Premium</t>
-  </si>
-  <si>
-    <t>HUD-IL 2002</t>
-  </si>
-  <si>
-    <t>07 13</t>
-  </si>
-  <si>
-    <t>Fully Earned Premium Endorsement</t>
-  </si>
-  <si>
-    <t>HUD-IL 2004</t>
-  </si>
-  <si>
-    <t>General Purpose Endorsement</t>
-  </si>
-  <si>
-    <t>HUD-IL 2005</t>
-  </si>
-  <si>
-    <t>Fifty Percent Earned Premium Endorsement</t>
-  </si>
-  <si>
-    <t>HUD NO 1005</t>
-  </si>
-  <si>
-    <t>12 21</t>
-  </si>
-  <si>
-    <t>California Policyholder Notice</t>
-  </si>
-  <si>
-    <t>CA</t>
+    <t>Exclusion - Wildfires</t>
+  </si>
+  <si>
+    <t>HXS-2042 (04-25)</t>
+  </si>
+  <si>
+    <t>all</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +130,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -214,7 +150,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -237,11 +173,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -256,6 +205,9 @@
     <xf numFmtId="47" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,7 +611,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" s="6">
         <v>41727</v>
@@ -668,13 +620,13 @@
         <v>2958101</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>15</v>
@@ -683,7 +635,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -695,332 +647,164 @@
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="6">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="5">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>16</v>
-      </c>
+      <c r="A3" s="5"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="5">
-        <v>15</v>
-      </c>
+      <c r="L3" s="5"/>
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="6">
-        <v>43871</v>
-      </c>
-      <c r="C4" s="6">
-        <v>2958465</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="A4" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="10">
+        <v>45912</v>
+      </c>
+      <c r="C4" s="10">
+        <v>2958101</v>
+      </c>
+      <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="5">
-        <v>1</v>
-      </c>
-      <c r="I4" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="F4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="5">
-        <v>31</v>
+      <c r="L4" s="9">
+        <v>735</v>
       </c>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="6">
-        <v>45608</v>
-      </c>
-      <c r="C5" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="5">
-        <v>1</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A5" s="5"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="5">
-        <v>50</v>
-      </c>
+      <c r="L5" s="5"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="6">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="5">
-        <v>1</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="5">
-        <v>60</v>
-      </c>
+      <c r="L6" s="5"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="6">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="5">
-        <v>1</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="5">
-        <v>70</v>
-      </c>
+      <c r="L7" s="5"/>
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="6">
-        <v>1</v>
-      </c>
-      <c r="C8" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="5">
-        <v>0</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
-      <c r="L8" s="5">
-        <v>80</v>
-      </c>
+      <c r="L8" s="5"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="7">
-        <v>43857</v>
-      </c>
-      <c r="C9" s="7">
-        <v>2958465</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="5">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A9" s="5"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
-      <c r="L9" s="5">
-        <v>83</v>
-      </c>
+      <c r="L9" s="5"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="6">
-        <v>1</v>
-      </c>
-      <c r="C10" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="A10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="5">
-        <v>85</v>
-      </c>
+      <c r="L10" s="5"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="6">
-        <v>44574</v>
-      </c>
-      <c r="C11" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" s="5">
-        <v>1</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="L11" s="5">
-        <v>10120</v>
-      </c>
+      <c r="A11" s="5"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="L11" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed script bugs and improved excel fields
</commit_message>
<xml_diff>
--- a/Rules/rules.xlsx
+++ b/Rules/rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JuanCoates\OneDrive - Combined Ratio\Desktop\forms script\PythonScript\Rules\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\Tools\Form_Files_Generator\PythonScript\Rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E5266F-2248-4879-9FA8-1C0F368D6F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B55064-09D7-47F8-B61D-46FFBF91515A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3510" yWindow="4095" windowWidth="19380" windowHeight="11175" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{A4EC016E-D811-43BC-B4EE-8E42B7F47CA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>FormNumber</t>
   </si>
@@ -65,49 +65,19 @@
     <t>FormType</t>
   </si>
   <si>
-    <t>ScribeTemplateID</t>
-  </si>
-  <si>
-    <t>PublicUrl</t>
-  </si>
-  <si>
     <t>DisplaySequence</t>
   </si>
   <si>
-    <t>P140XPath</t>
-  </si>
-  <si>
-    <t>FormConditionID</t>
-  </si>
-  <si>
-    <t>CommonGuid</t>
-  </si>
-  <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>IL 00 17</t>
-  </si>
-  <si>
-    <t>11 98</t>
-  </si>
-  <si>
-    <t>Common Policy Conditions</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Exclusion - Wildfires</t>
-  </si>
-  <si>
-    <t>HXS-2042 (04-25)</t>
-  </si>
-  <si>
-    <t>all</t>
+    <t>programid</t>
+  </si>
+  <si>
+    <t>products</t>
+  </si>
+  <si>
+    <t>lineOfBusiness</t>
+  </si>
+  <si>
+    <t>TransactionStatus</t>
   </si>
 </sst>
 </file>
@@ -174,16 +144,16 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -194,20 +164,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="47" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,111 +512,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5CE7AC6-E3FE-4E27-912C-E07231E907AF}">
-  <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="30.109375" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="1"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="6">
-        <v>41727</v>
-      </c>
-      <c r="C2" s="6">
-        <v>2958101</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="5">
-        <v>1</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="5">
-        <v>10</v>
-      </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -656,43 +604,31 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="7"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="10">
-        <v>45912</v>
-      </c>
-      <c r="C4" s="10">
-        <v>2958101</v>
-      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
       <c r="D4" s="5"/>
-      <c r="E4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>23</v>
-      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="8"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="9">
-        <v>735</v>
-      </c>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J4" s="5"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -702,14 +638,14 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="7"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -719,14 +655,14 @@
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="7"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -736,14 +672,14 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="7"/>
       <c r="L7" s="5"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -753,31 +689,31 @@
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="7"/>
       <c r="L8" s="5"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="7"/>
       <c r="L9" s="5"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -787,14 +723,14 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="7"/>
       <c r="L10" s="5"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -804,7 +740,29 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="7"/>
       <c r="L11" s="5"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>